<commit_message>
K-JAMDS_파라미터.xlsx 최신화 — 화면 설정 nocm·shpk, 엔진 기본 shoradCruiseExclusion·shoradPkRealism (서식 보존 갱신)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CW9SbhAbDs1WExRShGBGX4
</commit_message>
<xml_diff>
--- a/K-JAMDS_파라미터.xlsx
+++ b/K-JAMDS_파라미터.xlsx
@@ -311,7 +311,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>K-JAMDS 파라미터 참조본. 2026-09-30 현재 소스 fa0f5d3fbeed에서 재내보냈습니다. 엑셀 불러오기 기능은 없습니다.</x:v>
+        <x:v>K-JAMDS 파라미터 참조본. 2026-09-30 현재 소스 b61b500995b6에서 재내보냈습니다. 엑셀 불러오기 기능은 없습니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
@@ -42558,7 +42558,7 @@
       </x:c>
       <x:c r="B16" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">fa0f5d3fbeed</x:t>
+          <x:t xml:space="preserve">b61b500995b6</x:t>
         </x:is>
       </x:c>
       <x:c r="C16" s="3" t="inlineStr">
@@ -43148,37 +43148,37 @@
     <x:row r="54" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A54" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">화면 설정 lx</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B54" s="5">
+          <x:t xml:space="preserve">화면 설정 nocm</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B54">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C54" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">탄도 축선 발사점 연장 — 대표 사거리부터 비행, 탐지 선착이 기하에서 나옴 (ADR-091 · 이 화면만 기본 켜짐, 엔진 기본은 꺼짐). 적용 타입=boolean, 선언 기본값=1. 출처: prototype/command-flow.html PARAMS/파서</x:t>
+          <x:t xml:space="preserve">비호·천마 순항미사일 교전 제외 (ADR-107 ① · 이 화면만 기본 켜짐, 엔진 기본은 꺼짐). 적용 타입=boolean, 선언 기본값=1. 출처: prototype/command-flow.html PARAMS/파서</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="55" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A55" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">화면 설정 floor</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B55" s="5">
-        <x:v>0</x:v>
+          <x:t xml:space="preserve">화면 설정 shpk</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B55">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C55" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">C2 처리 시간 바닥 — 체계 처리 구간 + 운용자 판단을 따로 추첨, 평균 불변 (ADR-092 · 기본 꺼짐). 적용 타입=boolean, 선언 기본값=0. 출처: prototype/command-flow.html PARAMS/파서</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="56" ht="52.79999923706055" hidden="0" customHeight="1">
+          <x:t xml:space="preserve">비호·천마 소형 무인기·순항 요격확률을 WPN-SHORAD-PK-01(0.1/0.3/0.5)로 (ADR-107 ② · 이 화면만 기본 켜짐, 엔진 기본은 꺼짐). 적용 타입=boolean, 선언 기본값=1. 출처: prototype/command-flow.html PARAMS/파서</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A56" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">화면 설정 pipe</x:t>
+          <x:t xml:space="preserve">화면 설정 lx</x:t>
         </x:is>
       </x:c>
       <x:c r="B56" s="5">
@@ -43186,59 +43186,59 @@
       </x:c>
       <x:c r="C56" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">협조 파이프라인 현실화 — 실행가능 사수 있을 때만 협조 요청 · 회신은 협조 계선 역방향 · C2A 회신 처리 큐 (ADR-093 · 이 화면만 기본 켜짐, 엔진 기본은 꺼짐). 적용 타입=boolean, 선언 기본값=1. 출처: prototype/command-flow.html PARAMS/파서</x:t>
+          <x:t xml:space="preserve">탄도 축선 발사점 연장 — 대표 사거리부터 비행, 탐지 선착이 기하에서 나옴 (ADR-091 · 이 화면만 기본 켜짐, 엔진 기본은 꺼짐). 적용 타입=boolean, 선언 기본값=1. 출처: prototype/command-flow.html PARAMS/파서</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="57" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A57" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">화면 설정 icc</x:t>
+          <x:t xml:space="preserve">화면 설정 floor</x:t>
         </x:is>
       </x:c>
       <x:c r="B57" s="5">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C57" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">ICC 중계 인가 — 교전명령을 ICC가 접수·인가하고 권역 내 재배정/반송 (ADR-094 · 이 화면만 기본 켜짐, 엔진 기본은 꺼짐). 적용 타입=boolean, 선언 기본값=1. 출처: prototype/command-flow.html PARAMS/파서</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="58" ht="39.599998474121094" hidden="0" customHeight="1">
+          <x:t xml:space="preserve">C2 처리 시간 바닥 — 체계 처리 구간 + 운용자 판단을 따로 추첨, 평균 불변 (ADR-092 · 기본 꺼짐). 적용 타입=boolean, 선언 기본값=0. 출처: prototype/command-flow.html PARAMS/파서</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A58" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">화면 설정 iccsec</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B58">
-        <x:v>-1</x:v>
+          <x:t xml:space="preserve">화면 설정 pipe</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B58" s="5">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C58" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">ICC 중계 인가 시간(초) 민감도 — 미지정(-1)이면 ICC 기본 9초, 0이면 재검증 로직만 (ADR-094). 적용 타입=number, 선언 기본값=-1. 출처: prototype/command-flow.html PARAMS/파서</x:t>
+          <x:t xml:space="preserve">협조 파이프라인 현실화 — 실행가능 사수 있을 때만 협조 요청 · 회신은 협조 계선 역방향 · C2A 회신 처리 큐 (ADR-093 · 이 화면만 기본 켜짐, 엔진 기본은 꺼짐). 적용 타입=boolean, 선언 기본값=1. 출처: prototype/command-flow.html PARAMS/파서</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="59" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A59" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">화면 설정 ecs</x:t>
+          <x:t xml:space="preserve">화면 설정 icc</x:t>
         </x:is>
       </x:c>
       <x:c r="B59" s="5">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C59" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">ECS 실행 시간 ADSIM 정합 — 교전명령 실행을 10초로 (ADR-095 · 양 모드 공통 · 기본 꺼짐). 적용 타입=boolean, 선언 기본값=0. 출처: prototype/command-flow.html PARAMS/파서</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="60" ht="26.399999618530273" hidden="0" customHeight="1">
+          <x:t xml:space="preserve">ICC 중계 인가 — 교전명령을 ICC가 접수·인가하고 권역 내 재배정/반송 (ADR-094 · 이 화면만 기본 켜짐, 엔진 기본은 꺼짐). 적용 타입=boolean, 선언 기본값=1. 출처: prototype/command-flow.html PARAMS/파서</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A60" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">화면 설정 ecssec</x:t>
+          <x:t xml:space="preserve">화면 설정 iccsec</x:t>
         </x:is>
       </x:c>
       <x:c r="B60">
@@ -43246,119 +43246,119 @@
       </x:c>
       <x:c r="C60" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">ECS 실행 시간(초) 민감도 — 미지정(-1)이면 10초 (ADR-095). 적용 타입=number, 선언 기본값=-1. 출처: prototype/command-flow.html PARAMS/파서</x:t>
+          <x:t xml:space="preserve">ICC 중계 인가 시간(초) 민감도 — 미지정(-1)이면 ICC 기본 9초, 0이면 재검증 로직만 (ADR-094). 적용 타입=number, 선언 기본값=-1. 출처: prototype/command-flow.html PARAMS/파서</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="61" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A61" s="2" t="inlineStr">
         <x:is>
+          <x:t xml:space="preserve">화면 설정 ecs</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B61" s="5">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C61" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">ECS 실행 시간 ADSIM 정합 — 교전명령 실행을 10초로 (ADR-095 · 양 모드 공통 · 기본 꺼짐). 적용 타입=boolean, 선언 기본값=0. 출처: prototype/command-flow.html PARAMS/파서</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A62" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">화면 설정 ecssec</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B62">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="C62" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">ECS 실행 시간(초) 민감도 — 미지정(-1)이면 10초 (ADR-095). 적용 타입=number, 선언 기본값=-1. 출처: prototype/command-flow.html PARAMS/파서</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A63" s="2" t="inlineStr">
+        <x:is>
           <x:t xml:space="preserve">화면 설정 aim</x:t>
         </x:is>
       </x:c>
-      <x:c r="B61" s="5">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C61" s="3" t="inlineStr">
+      <x:c r="B63" s="5">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C63" s="3" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">표적 카탈로그 — 탄도탄이 조준점 10점을 나눠 노린다 (ADR-097 · 이 화면만 기본 켜짐, 엔진 기본은 꺼짐). 적용 타입=boolean, 선언 기본값=1. 출처: prototype/command-flow.html PARAMS/파서</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="62" ht="52.79999923706055" hidden="0" customHeight="1">
-      <x:c r="A62" s="3" t="inlineStr">
+    <x:row r="64" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A64" s="3" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">화면 설정 par</x:t>
         </x:is>
       </x:c>
-      <x:c r="B62" s="5">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C62" s="3" t="inlineStr">
+      <x:c r="B64" s="5">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C64" s="3" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">C2 결심 시간 동일화 — To-Be 결심 노드(IAOC) 운용자 판단 시간을 As-Is 결심 노드(KAMDOC·MCRC)와 같게 (ADR-099 · codex 정합 · 이 화면만 기본 켜짐, 엔진 기본은 꺼짐). 적용 타입=boolean, 선언 기본값=1. 출처: prototype/command-flow.html PARAMS/파서</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="63" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A63" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">화면 설정 issue</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B63" s="5">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C63" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">교전명령 발령 작업 — 결심 노드가 명령을 낼 때마다 큐를 탄다 (ADR-096 · 기본 꺼짐: ADSIM에는 없는 비용). 적용 타입=boolean, 선언 기본값=0. 출처: prototype/command-flow.html PARAMS/파서</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="64" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A64" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">화면 설정 issuesec</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B64">
-        <x:v>-1</x:v>
-      </x:c>
-      <x:c r="C64" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">발령 시간(초) 민감도 — 미지정(-1)이면 노드 체계 성분(KAMDOC 7.5·IAOC 1.5초) (ADR-096). 적용 타입=number, 선언 기본값=-1. 출처: prototype/command-flow.html PARAMS/파서</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="65" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A65" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">엔진 기본 highResolutionDeployment</x:t>
+          <x:t xml:space="preserve">화면 설정 issue</x:t>
         </x:is>
       </x:c>
       <x:c r="B65" s="5">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C65" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">features를 명시하지 않은 Simulation 생성값. 화면 전달값=true. 출처: js/engine/sim-engine.js</x:t>
+          <x:t xml:space="preserve">교전명령 발령 작업 — 결심 노드가 명령을 낼 때마다 큐를 탄다 (ADR-096 · 기본 꺼짐: ADSIM에는 없는 비용). 적용 타입=boolean, 선언 기본값=0. 출처: prototype/command-flow.html PARAMS/파서</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="66" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A66" s="3" t="inlineStr">
         <x:is>
+          <x:t xml:space="preserve">화면 설정 issuesec</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B66">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="C66" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">발령 시간(초) 민감도 — 미지정(-1)이면 노드 체계 성분(KAMDOC 7.5·IAOC 1.5초) (ADR-096). 적용 타입=number, 선언 기본값=-1. 출처: prototype/command-flow.html PARAMS/파서</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A67" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">엔진 기본 highResolutionDeployment</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B67" s="5">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C67" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">features를 명시하지 않은 Simulation 생성값. 화면 전달값=true. 출처: js/engine/sim-engine.js</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A68" s="3" t="inlineStr">
+        <x:is>
           <x:t xml:space="preserve">엔진 기본 threatTargetDispersion</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B66" s="5">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C66" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">features를 명시하지 않은 Simulation 생성값. 화면 전달값=true. 출처: js/engine/sim-engine.js</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="67" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A67" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">엔진 기본 southernAxes</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B67" s="5">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C67" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">features를 명시하지 않은 Simulation 생성값. 화면 전달값=true. 출처: js/engine/sim-engine.js</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="68" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A68" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">엔진 기본 linkSemanticsV2</x:t>
         </x:is>
       </x:c>
       <x:c r="B68" s="5">
@@ -43373,7 +43373,7 @@
     <x:row r="69" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A69" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">엔진 기본 sensorReportParity</x:t>
+          <x:t xml:space="preserve">엔진 기본 southernAxes</x:t>
         </x:is>
       </x:c>
       <x:c r="B69" s="5">
@@ -43385,10 +43385,10 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="70" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="70" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A70" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">엔진 기본 sawtoothFreshness</x:t>
+          <x:t xml:space="preserve">엔진 기본 linkSemanticsV2</x:t>
         </x:is>
       </x:c>
       <x:c r="B70" s="5">
@@ -43403,7 +43403,7 @@
     <x:row r="71" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A71" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">엔진 기본 approvalChain</x:t>
+          <x:t xml:space="preserve">엔진 기본 sensorReportParity</x:t>
         </x:is>
       </x:c>
       <x:c r="B71" s="5">
@@ -43418,7 +43418,7 @@
     <x:row r="72" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A72" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">엔진 기본 unifiedEngagementState</x:t>
+          <x:t xml:space="preserve">엔진 기본 sawtoothFreshness</x:t>
         </x:is>
       </x:c>
       <x:c r="B72" s="5">
@@ -43433,7 +43433,7 @@
     <x:row r="73" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A73" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">엔진 기본 selfDefenseFire</x:t>
+          <x:t xml:space="preserve">엔진 기본 approvalChain</x:t>
         </x:is>
       </x:c>
       <x:c r="B73" s="5">
@@ -43445,42 +43445,40 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="74" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="74" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A74" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">엔진 기본 engageOnRemote</x:t>
+          <x:t xml:space="preserve">엔진 기본 unifiedEngagementState</x:t>
         </x:is>
       </x:c>
       <x:c r="B74" s="5">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C74" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">features를 명시하지 않은 Simulation 생성값. 화면 전달값=false. 출처: js/engine/sim-engine.js</x:t>
+          <x:t xml:space="preserve">features를 명시하지 않은 Simulation 생성값. 화면 전달값=true. 출처: js/engine/sim-engine.js</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="75" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A75" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">엔진 기본 usfkTrackSharing</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B75" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">미지정</x:t>
-        </x:is>
+          <x:t xml:space="preserve">엔진 기본 selfDefenseFire</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B75" s="5">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C75" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">features를 명시하지 않은 Simulation 생성값. 화면 전달값=null. 출처: js/engine/sim-engine.js</x:t>
+          <x:t xml:space="preserve">features를 명시하지 않은 Simulation 생성값. 화면 전달값=true. 출처: js/engine/sim-engine.js</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="76" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A76" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">엔진 기본 wtaSuitability</x:t>
+          <x:t xml:space="preserve">엔진 기본 engageOnRemote</x:t>
         </x:is>
       </x:c>
       <x:c r="B76" s="5">
@@ -43492,25 +43490,27 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="77" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="77" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A77" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">엔진 기본 uavLocalSelfEngage</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B77" s="5">
-        <x:v>0</x:v>
+          <x:t xml:space="preserve">엔진 기본 usfkTrackSharing</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B77" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미지정</x:t>
+        </x:is>
       </x:c>
       <x:c r="C77" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">features를 명시하지 않은 Simulation 생성값. 화면 전달값=false. 출처: js/engine/sim-engine.js</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="78" ht="39.599998474121094" hidden="0" customHeight="1">
+          <x:t xml:space="preserve">features를 명시하지 않은 Simulation 생성값. 화면 전달값=null. 출처: js/engine/sim-engine.js</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A78" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">엔진 기본 earlyWarningReport</x:t>
+          <x:t xml:space="preserve">엔진 기본 wtaSuitability</x:t>
         </x:is>
       </x:c>
       <x:c r="B78" s="5">
@@ -43525,7 +43525,7 @@
     <x:row r="79" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A79" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">엔진 기본 ballisticReportSource</x:t>
+          <x:t xml:space="preserve">엔진 기본 uavLocalSelfEngage</x:t>
         </x:is>
       </x:c>
       <x:c r="B79" s="5">
@@ -43533,14 +43533,14 @@
       </x:c>
       <x:c r="C79" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">features를 명시하지 않은 Simulation 생성값. 화면 전달값=true. 출처: js/engine/sim-engine.js</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="80" ht="26.399999618530273" hidden="0" customHeight="1">
+          <x:t xml:space="preserve">features를 명시하지 않은 Simulation 생성값. 화면 전달값=false. 출처: js/engine/sim-engine.js</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A80" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">엔진 기본 standbyCue</x:t>
+          <x:t xml:space="preserve">엔진 기본 earlyWarningReport</x:t>
         </x:is>
       </x:c>
       <x:c r="B80" s="5">
@@ -43548,14 +43548,14 @@
       </x:c>
       <x:c r="C80" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">features를 명시하지 않은 Simulation 생성값. 화면 전달값=true. 출처: js/engine/sim-engine.js</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="81" ht="26.399999618530273" hidden="0" customHeight="1">
+          <x:t xml:space="preserve">features를 명시하지 않은 Simulation 생성값. 화면 전달값=false. 출처: js/engine/sim-engine.js</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A81" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">엔진 기본 commanderRouteRetry</x:t>
+          <x:t xml:space="preserve">엔진 기본 ballisticReportSource</x:t>
         </x:is>
       </x:c>
       <x:c r="B81" s="5">
@@ -43570,24 +43570,22 @@
     <x:row r="82" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A82" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">엔진 기본 rokUsfkCoordination</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B82" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">미지정</x:t>
-        </x:is>
+          <x:t xml:space="preserve">엔진 기본 standbyCue</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B82" s="5">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C82" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">features를 명시하지 않은 Simulation 생성값. 화면 전달값="voice". 출처: js/engine/sim-engine.js</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="83" ht="39.599998474121094" hidden="0" customHeight="1">
+          <x:t xml:space="preserve">features를 명시하지 않은 Simulation 생성값. 화면 전달값=true. 출처: js/engine/sim-engine.js</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A83" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">엔진 기본 ballisticLaunchAxes</x:t>
+          <x:t xml:space="preserve">엔진 기본 shoradCruiseExclusion</x:t>
         </x:is>
       </x:c>
       <x:c r="B83" s="5">
@@ -43602,7 +43600,7 @@
     <x:row r="84" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A84" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">엔진 기본 threatAimpoints</x:t>
+          <x:t xml:space="preserve">엔진 기본 shoradPkRealism</x:t>
         </x:is>
       </x:c>
       <x:c r="B84" s="5">
@@ -43614,10 +43612,10 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="85" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="85" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A85" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">엔진 기본 c2DecisionTimeParity</x:t>
+          <x:t xml:space="preserve">엔진 기본 commanderRouteRetry</x:t>
         </x:is>
       </x:c>
       <x:c r="B85" s="5">
@@ -43632,25 +43630,27 @@
     <x:row r="86" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A86" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">엔진 기본 c2ServiceFloor</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B86" s="7">
-        <x:v>0</x:v>
+          <x:t xml:space="preserve">엔진 기본 rokUsfkCoordination</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B86" s="5" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미지정</x:t>
+        </x:is>
       </x:c>
       <x:c r="C86" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">features를 명시하지 않은 Simulation 생성값. 화면 전달값=false. 출처: js/engine/sim-engine.js</x:t>
+          <x:t xml:space="preserve">features를 명시하지 않은 Simulation 생성값. 화면 전달값="voice". 출처: js/engine/sim-engine.js</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="87" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A87" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">엔진 기본 approvalPipelineRealism</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B87" s="7">
+          <x:t xml:space="preserve">엔진 기본 ballisticLaunchAxes</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B87" s="5">
         <x:v>0</x:v>
       </x:c>
       <x:c r="C87" s="3" t="inlineStr">
@@ -43659,13 +43659,13 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="88" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="88" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A88" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">엔진 기본 iccRelayAuthorization</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B88" s="7">
+          <x:t xml:space="preserve">엔진 기본 threatAimpoints</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B88" s="5">
         <x:v>0</x:v>
       </x:c>
       <x:c r="C88" s="3" t="inlineStr">
@@ -43674,25 +43674,25 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="89" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="89" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A89" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">엔진 기본 ecsExecutionTime</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B89" s="7">
+          <x:t xml:space="preserve">엔진 기본 c2DecisionTimeParity</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B89" s="5">
         <x:v>0</x:v>
       </x:c>
       <x:c r="C89" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">features를 명시하지 않은 Simulation 생성값. 화면 전달값=false. 출처: js/engine/sim-engine.js</x:t>
+          <x:t xml:space="preserve">features를 명시하지 않은 Simulation 생성값. 화면 전달값=true. 출처: js/engine/sim-engine.js</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="90" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A90" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">엔진 기본 directiveIssueTime</x:t>
+          <x:t xml:space="preserve">엔진 기본 c2ServiceFloor</x:t>
         </x:is>
       </x:c>
       <x:c r="B90" s="7">
@@ -43707,97 +43707,89 @@
     <x:row r="91" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A91" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SHA-256 js/config/system-types.js</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B91" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">c9b3efd9d9ed4de363745ede9b35eac3045ef1b1c0273ec489dd3c9074cbb262</x:t>
-        </x:is>
+          <x:t xml:space="preserve">엔진 기본 approvalPipelineRealism</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B91" s="7">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C91" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">작업 파일 내용 해시. 경로는 저장소 루트 기준</x:t>
+          <x:t xml:space="preserve">features를 명시하지 않은 Simulation 생성값. 화면 전달값=true. 출처: js/engine/sim-engine.js</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="92" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A92" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SHA-256 js/config/deployments.js</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B92" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">bb4ca552f32432da3a5b8374e7d0a7585f138c3e639f8b8ab5d6aa92831f89cf</x:t>
-        </x:is>
+          <x:t xml:space="preserve">엔진 기본 iccRelayAuthorization</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B92" s="7">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C92" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">작업 파일 내용 해시. 경로는 저장소 루트 기준</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="93" ht="39.599998474121094" hidden="0" customHeight="1">
+          <x:t xml:space="preserve">features를 명시하지 않은 Simulation 생성값. 화면 전달값=true. 출처: js/engine/sim-engine.js</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A93" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SHA-256 js/config/deployment-adapter.js</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B93" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">0d98a9a13251362a1408e525b7b643a6a1328ba80f4c09e5920d2c0b18a15a57</x:t>
-        </x:is>
+          <x:t xml:space="preserve">엔진 기본 ecsExecutionTime</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B93" s="7">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C93" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">작업 파일 내용 해시. 경로는 저장소 루트 기준</x:t>
+          <x:t xml:space="preserve">features를 명시하지 않은 Simulation 생성값. 화면 전달값=false. 출처: js/engine/sim-engine.js</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="94" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A94" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SHA-256 js/data/threats.js</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B94" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">155bd9ec551fd24488dffd8fbe2af0fec6e86b09b4b43641aa4e5d2e779d6047</x:t>
-        </x:is>
+          <x:t xml:space="preserve">엔진 기본 directiveIssueTime</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B94" s="7">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C94" s="3" t="inlineStr">
         <x:is>
+          <x:t xml:space="preserve">features를 명시하지 않은 Simulation 생성값. 화면 전달값=false. 출처: js/engine/sim-engine.js</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="95" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A95" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SHA-256 js/config/system-types.js</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B95" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">c9b3efd9d9ed4de363745ede9b35eac3045ef1b1c0273ec489dd3c9074cbb262</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C95" s="3" t="inlineStr">
+        <x:is>
           <x:t xml:space="preserve">작업 파일 내용 해시. 경로는 저장소 루트 기준</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="95" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A95" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SHA-256 js/data/axes.js</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B95" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">c05ca5f35b544b42d770adae4dc85fedaea526e00268bcb916915be6536eda8d</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C95" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">작업 파일 내용 해시. 경로는 저장소 루트 기준</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="96" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="96" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A96" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SHA-256 js/data/scenarios.js</x:t>
+          <x:t xml:space="preserve">SHA-256 js/config/deployments.js</x:t>
         </x:is>
       </x:c>
       <x:c r="B96" s="3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">e0d14eb11a8488ca646dbede9700c794eea4b878d6b9bf65ab6807745230c92f</x:t>
+          <x:t xml:space="preserve">bb4ca552f32432da3a5b8374e7d0a7585f138c3e639f8b8ab5d6aa92831f89cf</x:t>
         </x:is>
       </x:c>
       <x:c r="C96" s="3" t="inlineStr">
@@ -43809,66 +43801,134 @@
     <x:row r="97" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A97" s="3" t="inlineStr">
         <x:is>
+          <x:t xml:space="preserve">SHA-256 js/config/deployment-adapter.js</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B97" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">0d98a9a13251362a1408e525b7b643a6a1328ba80f4c09e5920d2c0b18a15a57</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C97" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">작업 파일 내용 해시. 경로는 저장소 루트 기준</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="98" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A98" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SHA-256 js/data/threats.js</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B98" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">155bd9ec551fd24488dffd8fbe2af0fec6e86b09b4b43641aa4e5d2e779d6047</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C98" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">작업 파일 내용 해시. 경로는 저장소 루트 기준</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A99" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SHA-256 js/data/axes.js</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B99" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">c05ca5f35b544b42d770adae4dc85fedaea526e00268bcb916915be6536eda8d</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C99" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">작업 파일 내용 해시. 경로는 저장소 루트 기준</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="100" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A100" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SHA-256 js/data/scenarios.js</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B100" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">e0d14eb11a8488ca646dbede9700c794eea4b878d6b9bf65ab6807745230c92f</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C100" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">작업 파일 내용 해시. 경로는 저장소 루트 기준</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="101" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A101" s="3" t="inlineStr">
+        <x:is>
           <x:t xml:space="preserve">SHA-256 js/engine/sim-engine.js</x:t>
         </x:is>
       </x:c>
-      <x:c r="B97" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">65b84d17b5e7f562d3c06ef8915b71a6f9cec55f77a0124885f55b6ccf3fe7e1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C97" s="3" t="inlineStr">
+      <x:c r="B101" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">f31727fbef3bfe129f113c93216b7d65e207eaafc3aeb9de7ea4f1b21106cef2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C101" s="3" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">작업 파일 내용 해시. 경로는 저장소 루트 기준</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="98" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A98" s="3" t="inlineStr">
+    <x:row r="102" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A102" s="3" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">SHA-256 js/model/iads/c2-agent.js</x:t>
         </x:is>
       </x:c>
-      <x:c r="B98" s="3" t="inlineStr">
+      <x:c r="B102" s="3" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">d697f803fbf208fcaa952c26ab81720d227b00a6c7592d1025b6cffcb12b5d6f</x:t>
         </x:is>
       </x:c>
-      <x:c r="C98" s="3" t="inlineStr">
+      <x:c r="C102" s="3" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">작업 파일 내용 해시. 경로는 저장소 루트 기준</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="99" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A99" s="3" t="inlineStr">
+    <x:row r="103" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A103" s="3" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">SHA-256 prototype/command-flow.html</x:t>
         </x:is>
       </x:c>
-      <x:c r="B99" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">bf21e5188dcfb56d7d13e52b7882fe22354b7a5542e6a8fedb6dd43682c12ec3</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C99" s="3" t="inlineStr">
+      <x:c r="B103" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">7e7857571866f075d0b64f3146714e8718925b9b6c981d70c392809119d73d83</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C103" s="3" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">작업 파일 내용 해시. 경로는 저장소 루트 기준</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="100" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A100" s="3" t="inlineStr">
+    <x:row r="104" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A104" s="3" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">SHA-256 scripts/export-params-xlsx.mjs</x:t>
         </x:is>
       </x:c>
-      <x:c r="B100" s="3" t="inlineStr">
+      <x:c r="B104" s="3" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">65edfc580d2ac6dd0e9aa95587af182dc5749126d61f672f0533f4ff8c5220f6</x:t>
         </x:is>
       </x:c>
-      <x:c r="C100" s="3" t="inlineStr">
+      <x:c r="C104" s="3" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">작업 파일 내용 해시. 경로는 저장소 루트 기준</x:t>
         </x:is>

</xml_diff>